<commit_message>
Improve DAP table generation: filter indicators by survey usage, skip calculate types and "00" codes, lookup indicator bank rows by code, and clean output columns
- Rewrite `..construct_dap_rows` to match indicator bank rows via indicator_code/dep_indicator_code and skip rows lacking research questions or labels
- Simplify `iphra_dap_flextable` with proportional column widths and renamed headers
- Make DAP section headers conditional on tool params and remove Annex 1
- Update reference indicator bank, household tool, and test TOR resources
- Expand objective codes in manual protocol workflow test
</commit_message>
<xml_diff>
--- a/inst/resources/reference_indicator_bank.xlsx
+++ b/inst/resources/reference_indicator_bank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\Positron\public_health_resources\inst\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCB0968C-A523-4925-868B-696C113DECB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA07700E-2BCA-4D4E-9B43-017FA16CFC78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A81D9A7-8734-4191-8BBE-89A5AF7A65A9}"/>
+    <workbookView xWindow="-14970" yWindow="120" windowWidth="14955" windowHeight="15360" xr2:uid="{4A81D9A7-8734-4191-8BBE-89A5AF7A65A9}"/>
   </bookViews>
   <sheets>
     <sheet name="indicator_bank" sheetId="2" r:id="rId1"/>
@@ -3228,6 +3228,9 @@
       <c r="C2" s="2">
         <v>10101</v>
       </c>
+      <c r="D2" s="2">
+        <v>10000</v>
+      </c>
       <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
@@ -3272,6 +3275,9 @@
       <c r="C3" s="2">
         <v>10102</v>
       </c>
+      <c r="D3" s="2">
+        <v>10000</v>
+      </c>
       <c r="E3" s="2" t="s">
         <v>7</v>
       </c>
@@ -3316,6 +3322,9 @@
       <c r="C4" s="2">
         <v>10103</v>
       </c>
+      <c r="D4" s="2">
+        <v>10102</v>
+      </c>
       <c r="E4" s="2" t="s">
         <v>7</v>
       </c>
@@ -3403,6 +3412,9 @@
       </c>
       <c r="C6" s="2">
         <v>10105</v>
+      </c>
+      <c r="D6" s="2">
+        <v>10000</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>7</v>

</xml_diff>